<commit_message>
feat: Enhance question management by supporting up to 8 answers and improving import validation
</commit_message>
<xml_diff>
--- a/admin/public/templates/mau_import.xlsx
+++ b/admin/public/templates/mau_import.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Questions" sheetId="1" r:id="R389f17fe4c774224"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Questions" sheetId="1" r:id="R24e47c790ba24fef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32,7 +32,7 @@
       <x:name val="Calibri"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -42,6 +42,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFD7E4BC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -89,7 +94,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="19">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
@@ -124,6 +129,17 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -134,17 +150,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="QuestionImportTemplate" displayName="QuestionImportTemplate" ref="A1:I4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="9">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="QuestionImportTemplate" displayName="QuestionImportTemplate" ref="A1:M4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="13">
     <x:tableColumn id="1" name="Nội dung câu hỏi"/>
     <x:tableColumn id="2" name="Độ khó"/>
     <x:tableColumn id="3" name="Đáp án A"/>
     <x:tableColumn id="4" name="Đáp án B"/>
     <x:tableColumn id="5" name="Đáp án C"/>
     <x:tableColumn id="6" name="Đáp án D"/>
-    <x:tableColumn id="7" name="Đáp án đúng"/>
-    <x:tableColumn id="8" name="Ảnh/URL"/>
-    <x:tableColumn id="9" name="Loại câu hỏi"/>
+    <x:tableColumn id="7" name="Đáp án E"/>
+    <x:tableColumn id="8" name="Đáp án F"/>
+    <x:tableColumn id="9" name="Đáp án G"/>
+    <x:tableColumn id="10" name="Đáp án H"/>
+    <x:tableColumn id="11" name="Đáp án đúng"/>
+    <x:tableColumn id="12" name="Ảnh/URL"/>
+    <x:tableColumn id="13" name="Loại câu hỏi"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -369,41 +389,57 @@
     <x:col min="1" max="1" width="37.5" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="11.880000114440918" hidden="0" customWidth="1"/>
     <x:col min="3" max="6" width="25.7109375" customWidth="1"/>
-    <x:col min="7" max="7" width="11.880000114440918" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="27.5" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="13.130000114440918" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18.75" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="12" t="str">
+      <x:c r="A1" s="14" t="str">
         <x:v>Nội dung câu hỏi</x:v>
       </x:c>
-      <x:c r="B1" s="12" t="str">
+      <x:c r="B1" s="14" t="str">
         <x:v>Độ khó</x:v>
       </x:c>
-      <x:c r="C1" s="12" t="str">
+      <x:c r="C1" s="14" t="str">
         <x:v>Đáp án A</x:v>
       </x:c>
-      <x:c r="D1" s="12" t="str">
+      <x:c r="D1" s="14" t="str">
         <x:v>Đáp án B</x:v>
       </x:c>
-      <x:c r="E1" s="12" t="str">
+      <x:c r="E1" s="14" t="str">
         <x:v>Đáp án C</x:v>
       </x:c>
-      <x:c r="F1" s="12" t="str">
+      <x:c r="F1" s="14" t="str">
         <x:v>Đáp án D</x:v>
       </x:c>
-      <x:c r="G1" s="12" t="str">
+      <x:c r="G1" s="14" t="str">
+        <x:v>Đáp án E</x:v>
+      </x:c>
+      <x:c r="H1" s="15" t="str">
+        <x:v>Đáp án F</x:v>
+      </x:c>
+      <x:c r="I1" s="15" t="str">
+        <x:v>Đáp án G</x:v>
+      </x:c>
+      <x:c r="J1" s="15" t="str">
+        <x:v>Đáp án H</x:v>
+      </x:c>
+      <x:c r="K1" s="15" t="str">
         <x:v>Đáp án đúng</x:v>
       </x:c>
-      <x:c r="H1" s="13" t="str">
+      <x:c r="L1" s="15" t="str">
         <x:v>Ảnh/URL</x:v>
       </x:c>
-      <x:c r="I1" s="13" t="str">
+      <x:c r="M1" s="15" t="str">
         <x:v>Loại câu hỏi</x:v>
       </x:c>
     </x:row>
@@ -426,11 +462,15 @@
       <x:c r="F2" s="11" t="str">
         <x:v>$2$</x:v>
       </x:c>
-      <x:c r="G2" s="11" t="str">
+      <x:c r="G2" s="11" t="str"/>
+      <x:c r="H2" s="11" t="str"/>
+      <x:c r="I2" s="11" t="str"/>
+      <x:c r="J2" s="11" t="str"/>
+      <x:c r="K2" s="11" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="H2" s="11" t="str"/>
-      <x:c r="I2" s="11" t="str">
+      <x:c r="L2" s="11" t="str"/>
+      <x:c r="M2" s="11" t="str">
         <x:v>SINGLE_CHOICE</x:v>
       </x:c>
     </x:row>
@@ -454,10 +494,16 @@
         <x:v>Markdown hỗ trợ **in đậm**</x:v>
       </x:c>
       <x:c r="G3" s="11" t="str">
-        <x:v>ACD</x:v>
+        <x:v>Có thể thêm đáp án E</x:v>
       </x:c>
       <x:c r="H3" s="11" t="str"/>
-      <x:c r="I3" s="11" t="str">
+      <x:c r="I3" s="11" t="str"/>
+      <x:c r="J3" s="11" t="str"/>
+      <x:c r="K3" s="11" t="str">
+        <x:v>ACDE</x:v>
+      </x:c>
+      <x:c r="L3" s="11" t="str"/>
+      <x:c r="M3" s="11" t="str">
         <x:v>MULTIPLE_CHOICE</x:v>
       </x:c>
     </x:row>
@@ -480,13 +526,17 @@
       <x:c r="F4" s="11" t="str">
         <x:v>$S=ab$</x:v>
       </x:c>
-      <x:c r="G4" s="11" t="str">
+      <x:c r="G4" s="11" t="str"/>
+      <x:c r="H4" s="11" t="str"/>
+      <x:c r="I4" s="11" t="str"/>
+      <x:c r="J4" s="11" t="str"/>
+      <x:c r="K4" s="11" t="str">
         <x:v>A</x:v>
       </x:c>
-      <x:c r="H4" s="11" t="str">
+      <x:c r="L4" s="11" t="str">
         <x:v>images/circle.png</x:v>
       </x:c>
-      <x:c r="I4" s="11" t="str">
+      <x:c r="M4" s="11" t="str">
         <x:v>SINGLE_CHOICE</x:v>
       </x:c>
     </x:row>
@@ -501,7 +551,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R95fe2c6f277f4b15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8ad81a0dbb42441f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>